<commit_message>
not valid line break fix
</commit_message>
<xml_diff>
--- a/output/opodesh-test/book-output.xlsx
+++ b/output/opodesh-test/book-output.xlsx
@@ -507,8 +507,7 @@
 &lt;ar&gt;يَوْمَ تَشْهَدُ عَلَيْهِمْ أَلْسِنَتُهُمْ وَأَيْدِيهِمْ وَأَرْجُلُهُمْ بِمَا كَانُوا يَعْمَلُوْনَ&lt;/ar&gt;
 &lt;p&gt;'যেদিন তাদের বিরুদ্ধে সাক্ষ্য দিবে তাদের যবান, তাদের হাত ও তাদের পা তাদের কৃতকর্ম সম্বন্ধে' (আন-নূর, ২৪/২৪)।&lt;/p&gt;
 &lt;ar&gt;وَيَوْمَ يُحْশَرُ أَعْدَاءُ اللهِ إِلَى النَّارِ فَهُمْ يُوزَعُوْنَ إِذَا مَا جَاءُوهَا شَهِدَ عَلَيْهِمْ سَمْعُكُمْ وَأَبْصَارُكُمْ وَجُلُودُكُمْ بِمَا كَانُوا يَعْمَلُوْনَ وَقَالُوا لِجُلُوْدِهِمْ لِمَ شَهِدْتُمْ عَلَيْنَا قَالُوْا أَنْطَقَنَا اللَّهُ الَّذِي أَنْطَقَ كُلَّ شَيْءٍ وَهُوَ خَلَقَكُمْ أَوَّلَ مَرَّةٍ وَإِلَيْهِ تُرْجَعُوْنَ وَمَا كُنْتُمْ تَسْتَتِرُوْنَ أَنْ يَشْهَدَ عَلَيْكُمْ سَمْعُكُمْ وَلَا أَبْصَارُكُمْ وَلَا جُلُودُكُمْ وَلَكِنْ ظَنَنْتُمْ أَنَّ اللَّهَ لَا يَعْلَمُ كَثِيرًا مِمَّا تَعْمَلُوْনَ&lt;/ar&gt;
-&lt;p&gt;'যেদিন আল্লাহর শত্রুদের জাহান্নাম অভিমুখে সমবেত করা হবে, সেদিন তাদের তাড়িয়ে নিয়ে যাওয়া হবে বিভিন্ন দলে। পরিশেষে যখন তারা জাহান্নামের সন্নিকটে পৌঁছবে তখন তাদের কর্ণ, চক্ষু ও ত্বক (চামড়া) তাদের কৃতকর্ম সম্বন্ধে সাক্ষ্য দিবে। জাহান্নামীরা তাদের ত্বককে জিজ্ঞাসা করবে, তোমরা আমাদের বিরুদ্ধে সাক্ষ্য দিচ্ছ কেন? উত্তরে তারা বলবে, আল্লাহ যিনি সবকিছুকে বাকশক্তি&lt;/p&gt;
-&lt;p&gt;দিয়েছেন তিনি আমাদেরও বাকশক্তি দিয়েছেন। তিনি তোমাদের সৃষ্টি করেছেন প্রথম বার এবং তাঁরই নিকট তোমরা প্রত্যাবর্তিত হবে। তোমরা কিছু গোপন করতে না এই বিশ্বাসে যে, তোমাদের কর্ণ, চক্ষু এবং ত্বক তোমাদের বিরুদ্ধে সাক্ষ্য দিবে না। উপরন্তু তোমরা মনে করতে যে, তোমরা যা করতে তার অনেক কিছুই আল্লাহ জানেন না' (ফুছছিলাত, ৪১/১৯-২২)।&lt;/p&gt;
+&lt;p&gt;'যেদিন আল্লাহর শত্রুদের জাহান্নাম অভিমুখে সমবেত করা হবে, সেদিন তাদের তাড়িয়ে নিয়ে যাওয়া হবে বিভিন্ন দলে। পরিশেষে যখন তারা জাহান্নামের সন্নিকটে পৌঁছবে তখন তাদের কর্ণ, চক্ষু ও ত্বক (চামড়া) তাদের কৃতকর্ম সম্বন্ধে সাক্ষ্য দিবে। জাহান্নামীরা তাদের ত্বককে জিজ্ঞাসা করবে, তোমরা আমাদের বিরুদ্ধে সাক্ষ্য দিচ্ছ কেন? উত্তরে তারা বলবে, আল্লাহ যিনি সবকিছুকে বাকশক্তি দিয়েছেন তিনি আমাদেরও বাকশক্তি দিয়েছেন। তিনি তোমাদের সৃষ্টি করেছেন প্রথম বার এবং তাঁরই নিকট তোমরা প্রত্যাবর্তিত হবে। তোমরা কিছু গোপন করতে না এই বিশ্বাসে যে, তোমাদের কর্ণ, চক্ষু এবং ত্বক তোমাদের বিরুদ্ধে সাক্ষ্য দিবে না। উপরন্তু তোমরা মনে করতে যে, তোমরা যা করতে তার অনেক কিছুই আল্লাহ জানেন না' (ফুছছিলাত, ৪১/১৯-২২)।&lt;/p&gt;
 &lt;p&gt;হাদীছে এসেছে,&lt;/p&gt;
 &lt;ar&gt;عَنِ ابْنِ عُمَرَ قَالَ قَالَ رَسُولُ اللهِ ﷺ إِنَّ اللهَ يُدْنِي الْمُؤْمِنَ فَيَضَعُ عَلَيْهِ كَنَفَهُ، وَيَسْتُرُهُ فَيَقُولُ أَتَعْرِفُ ذَنْبَ كَذَا أَتَعْرِفُ ذَنْبَ كَذَا فَيَقُولُ نَعَمْ أَيْ رَبِّ . حَتَّى إِذَا قَرَّرَهُ بِذُنُوبِهِ وَرَأَى فِي نَفْسِهِ أَنَّهُ هَلَكَ قَالَ سَتَرْتُهَا عَلَيْكَ فِي الدُّنْيَا، وَأَنَا أَغْفِرُهَا لَكَ الْيَوْمَ ، فَيُعْطَى كِتَابَ حَسَنَاتِهِ، وَأَمَّا الْكَافِرُ وَالْمُنَافিقُونَ فَيَقُولُ الْأَشْهَادُ هَؤُلَاءِ الَّذِينَ كَذَبُوا عَلَى رَبِّهِمْ، أَلَا لَعْنَةُ اللَّهِ عَلَى الظَّالِمِينَ » .&lt;/ar&gt;
 &lt;p&gt;ইবনু উমার (রাঃ) বলেন, রাসূলুল্লাহ (ﷺ) বলেছেন, '(কিয়ামতের দিন) আল্লাহ তাআলা মুমিনদের নিজের নিকটবর্তী করবেন এবং আল্লাহ তাআলা নিজ বাজু তার উপরে রেখে তাকে ঢেকে নিবেন। অতঃপর আল্লাহ সেই বান্দাকে বলবেন, আচ্ছা! বলো দেখি, এই গুনাহটি তুমি করেছ কি? এই গুনাহটি সম্পর্কে তুমি অবগত আছ কি? সে বলবে হ্যাঁ, হে আমার রব! আমি অবগত আছি। শেষ পর্যন্ত এক একটি করে তার কৃত সমস্ত গুনাহের স্বীকৃতি আদায় করবেন। এদিকে সে বান্দা মনে মনে এই ধারণা করবে যে, সে এই সমস্ত অপরাধের কারণে নিশ্চিত ধ্বংস হবে। তখন আল্লাহ তাআলা বলবেন, দুনিয়াতে আমি তোমার এই সমস্ত অপরাধ ঢেকে রেখেছিলাম। আর আজ আমি তা মাফ করে দিব। অতঃপর তাকে নেকীর আমলনামা দেওয়া হবে। আর কাফের ও মুনাফেকদের সমস্ত সৃষ্টির সম্মুখে আনয়ন করা হবে এবং উচ্চৈস্বরে এই ঘোষণা দেওয়া হবে- এরা তারা, যারা স্বীয় পরওয়ারদিগারের বিরুদ্ধে মিথ্যারোপ করত। জেনে রাখ, এই সমস্ত জালেমদের উপর আজ আল্লাহর লানত' (ছহীহ বুখারী, হা/২৪৪১; ছহীহ মুসলিম, হা/২৭৬৮; মিশকাত, হা/৫৫৫১)।&lt;/p&gt;
@@ -516,12 +515,10 @@
 &lt;p&gt;আনাস (রাঃ) হতে বর্ণিত, তিনি বলেন, আমরা রাসূলুল্লাহ (ﷺ)-এর কাছে ছিলাম, হঠাৎ তিনি হাসলেন। অতঃপর জিজ্ঞাসা করলেন, তোমরা কি জান আমি কেন হাসছি? আমরা বললাম, আল্লাহ এবং তাঁর রাসূলই ভালো জানেন। তিনি বললেন, কিয়ামতের দিন বান্দা যে তার রবের সাথে সরাসরি কথা বলবে, সেই কথাটি স্মরণ করে হাসছি। বান্দা বলবে, হে রব! তুমি কি আমাকে জুলুম হতে নিরাপত্তা দান করনি? আল্লাহ বলবেন, হ্যাঁ, তখন বান্দা বলবে, আজ আমি আমার সম্পর্কে আপনজন ব্যতীত আমার বিরুদ্ধে অন্য কারো সাক্ষ্য গ্রহণ করব না। তখন আল্লাহ বলবেন, আজ তুমি নিজেই তোমার সাক্ষী হিসাবে এবং কিরামান-কাতেবীনের সাক্ষ্যই তোমার জন্য যথেষ্ট। অতঃপর আল্লাহ তাআলা তার মুখের উপর মোহর লাগিয়ে দিবেন এবং অঙ্গ-প্রত্যঙ্গকে বলা হবে, তোমরা কে কখন কী কী কাজ করেছ বলো। তখন অঙ্গ-প্রত্যঙ্গসমূহ তাদের কৃতকর্মসমূহ প্রকাশ করে দিবে। এরপর তার মুখকে স্বাভাবিক অবস্থায় খুলে দেওয়া হবে। তখন সে স্বীয় অঙ্গসমূহকে লক্ষ্য করে আক্ষেপের সাথে বলবে, হে দুর্ভাগা অঙ্গসমূহ! তোরা দূর হ! তোদের ধ্বংস হৌক! তোদের জন্যই তো আমি আমার রবের সাথে ঝগড়া করেছিলাম' (ছহীহ মুসলিম, হা/২৯৬৯; মিশকাত, হা/৫৫৫৪)।&lt;/p&gt;
 &lt;ar&gt;عَنْ أَبِي هُرَيْرَةَ قَالَ: قَالُوا : يَا رَسُولَ اللهِ! هَلْ نَرَى رَبَّنَا يَوْمَ الْقِيَامَةِ؟ قَالَ: هَلْ تُضَارُّونَ فِي رؤْيَةِ الشَّمْسِ فِي الظَّهِيرَةِ لَيْسَتْ فِي سَحَابَةٍ؟ قَالُوا: لَا ، قَالَ: فَهَلْ تُضَارُّونَ فِي رُؤْيَةِ الْقَمَرِ لَيْلَةَ الْبَدْرِ لَيْسَتْ فِي سَحَابَةٍ؟ قَالُوا : لَا. قَالَ: فَوَالَّذِي نَفْسِي بِيَدِهِ لَا تُضَارُّونَ فِي رُؤْيَةِ رَبِّكُمْ إِلَّا كَمَا تُضَارُّونَ فِي رُؤْيَةِ أَحَدِهِمَا. قَالَ: فَيَلْقَى الْعَبْدَ فَيَقُولُ: أَيْ قُلْ: أَلَمْ أُكْرِمْكَ وَأُسَوَّدْكَ وَأَزَوَّجْكَ، وَأُسَخَّرْ لَكَ الْخَيْلَ وَالْإِبِلَ ، وَأَذَرْكَ تَرْأَسُ وَتَرْبَعُ؟ فَيَقُولُ: بَلَى. قَالَ: فَيَقُولُ: أَفَظَنَنْتَ أَنَّكَ مُلَاقِي؟ فَيَقُولُ لَا فَيَقُولُ: فَإِنِّي قَدْ أَنْسَاكَ كَمَا نَسِيتَنِي. ثُمَّ يَلْقَى الثَّانِي فَذَكَرَ مِثْلَهُ ، ثُمَّ يَلْقَى الثَّالِثَ فَيَقُولُ لَهُ مِثْلَ ذَلِكَ، فَيَقُولُ: يَا رَبِّ آمَنْتُ بِكَ، وَبِكِতَابِكَ وَبِرُسُلِكَ، وَصَلَّيْتُ وَصُمْتُ، وَتَصَدَّقْتُ، وَيُثْنِي بِخَيْرٍ مَا اسْتَطَاعَ، يَقُولُ: هَاهُنَا إِذًا، ثُمَّ يُقَالُ: الْآنَ نَبْعَثُ شَاهِدًا عَلَيْكَ، وَيَتَفَكَّرُ فِي نَفْسِهِ: مَنْ ذَا الَّذِي يَشْهَدُ عَلَيَّ? فَيُخْتَمُ عَلَى فِيهِ وَيُقَالُ لِفَخِذِهِ: انْطِقِي؛ فَتَنْطِقُ فَخِذُهُ وَلَحْمُهُ وَعِظَامُهُ بِعَمَلِهِ، وَذَلِكَ لِيُعْذِرَ مِنْ نَفْسِهِ، وَذَلِكَ الْمُنَافِقُ، وَذَلِكَ الَّذِي سَخِطَ اللهُ عَلَيْهِ» .&lt;/ar&gt;
 &lt;p&gt;আবূ হুরায়রা (রাঃ) হতে বর্ণিত, তিনি বলেন, ছাহাবীগণ (রাঃ) বললেন, হে আল্লাহর রাসূল (ﷺ)! কিয়ামতের দিন কী আমরা আমাদের রবকে দেখতে পাব? তিনি বললেন, দ্বিপ্রহরে মেঘমুক্ত আকাশে সূর্য দেখতে কি তোমাদের মধ্যে পরস্পরে বাধা সৃষ্টি হয়? তারা বললেন, না। তিনি আরও বললেন, মেঘমুক্ত আকাশে পূর্ণিমার রাত্রে পূর্ণ চাঁদ দেখতে কি তোমাদের কোনো প্রকারের অসুবিধা হয়? তারা বললেন, না। অতঃপর তিনি বললেন, সেই মহান সত্তার কসম, যাঁর হাতে আমার প্রাণ! এই দুটির কোনো একটিকে দেখতে তোমাদের যেই পরিমাণ অসুবিধা হয়, সেই দিন তোমাদের রবকে দেখতে সেই পরিমাণ অসুবিধাও হবে না। এরপর রাসূল (ﷺ) বললেন, তখন আল্লাহ তাআলা কোনো এক বান্দাকে লক্ষ্য করে বলবেন, হে অমুক! আমি কি তোমাকে মর্যাদা দান করিনি? আমি কি তোমাকে সর্দারী দান করিনি? আমি কি তোমাকে বিবি দান করিনি? আমি কি তোমার জন্য ঘোড়া ও উটকে অনুগত করে দেয়নি? আমি কি তোমাকে এই সুযোগ দেয়নি যে, তুমি নিজ সম্প্রদায়ের নেতৃত্ব দিবে এবং তাদের নিকট হতে এক-চতুর্থাংশ মাল ভোগ করবে? জবাবে বান্দা বলবে, হ্যাঁ, (হে আমার প্রতিপালক!)। অতঃপর রাসূল (ﷺ) বলেন, তখন আল্লাহ তাআলা বান্দাকে বলবেন, আচ্ছা বলো দেখি, তোমার কি এই ধারণা ছিল যে, তুমি আমার সাক্ষাৎ লাভ করবে? বান্দা বলবে, না। এইবার আল্লাহ বলবেন, (দুনিয়াতে) তুমি যেভাবে আমাকে ভুলে গিয়েছিলে আজ আমিও (আখেরাতে) অনুরূপভাবে তোমাকে ভুলে থাকব। (অর্থাৎ তোমাকে আযাবে লিপ্ত রাখব)। অতঃপর আল্লাহ তাআলা দ্বিতীয় এক ব্যক্তিকে জিজ্ঞাসা করবেন, সেও অনুরূপ বলবে। তারপর তৃতীয় এক ব্যক্তির সাথে সাক্ষাৎ করবেন এবং তাকেও অনুরূপ কথা জিজ্ঞাসা করলে সে বলবে, হে আমার প্রতিপালক! আমি তোমার প্রতি, তোমার কিতাবের প্রতি এবং তোমার সমস্ত নবীগণের প্রতি ঈমান এনেছি, ছালাত আদায় করেছি, ছিয়াম পালন করেছি এবং দান-ছাদাকা করেছি। মোটকথা, সে সাধ্য পরিমাণ নিজের নেক কার্যসমূহের একটি তালিকা আল্লাহর সম্মুখে তুলে ধরবে। তখন আল্লাহ তাআলা বলবেন, আচ্ছা! তুমি তো তোমার কথা বললে, এখন এখানেই দাঁড়াও, এক্ষুণি তোমার ব্যাপারে সাক্ষী উপস্থিত করছি। এই কথা শুনে বান্দা মনে মনে চিন্তা করবে, এমন কে আছে যে, এখানে আমার বিরুদ্ধে সাক্ষ্য দিবে? অতঃপর তার মুখে মোহর লাগিয়ে দেওয়া হবে এবং তার রানকে বলা হবে, তুমি বলো, তখন তার রান, হাড়, মাংস প্রভৃতি এক একটি করে বলে ফেলবে, এরা যা যা করেছিল। তার মুখে মোহর লাগিয়ে অঙ্গ-প্রত্যঙ্গ হতে এই জন্য সাক্ষী গ্রহণ করা হবে, যেন সেই বান্দা কোনো ওযর-আপত্তি পেশ করতে না পারে। বস্তুত যেই বান্দার কথা আলোচনা করা হয়েছে, সে হলো মুনাফেক এবং এই কারণেই আল্লাহ তার প্রতি অত্যন্ত ক্ষুব্ধ হবেন (ছহীহ মুসলিম, হা/২৯৬৮; মিশকাত, হা/৫৫৫৫)।&lt;/p&gt;
-&lt;ar&gt;عَنْ عَبْدِ اللَّهِ بْنِ عَمْرٍو قَالَ: قَالَ رَسُولُ اللهِ ﷺ : «إِنَّ اللَّهَ سَيُخَلَّصُ رَجُلًا مِنْ أُمَّتِي عَلَى رُءُوسِ الْخَلَائِقِ يَوْمَ الْقِيَامَةِ، فَيَنْشُرُ عَلَيْهِ تِسْعَةً وَتِسْعِينَ سِجِلًا، كُلُّ سِجِلٌ مِثْلَ مَدَّ الْبَصَرِ ، ثُمَّ يَقُولُ أَتُنْكِرُ مِنْ هَذَا شَيْئًا أَظْلَمَكَ كَتَبَتِي الْحَافِظُونَ؟ فَيَقُولُ: لَا يَا رَبِّ فَيَقُولُ: أَفَلَكَ عُذْرُ؟ قَالَ: لَا يَا رَبِّ فَيَقُولُ : بَلَى؛ إِنَّ لَكَ عِنْدَنَا حَسَنَةً، وَإِنَّهُ لَا ظُلْمَ عَلَيْكَ الْيَوْمَ، فَتُخْرَجُ بِطَاقَةٌ فِيهَا: أَشْهَدُ أَنْ لَا إِلَهَ إِلَّا اللهُ، وَأَنَّ مُحَمَّدًا عَبْدُهُ وَرَسُولُهُ، فَيَقُولُ: احْضُرْ&lt;/ar&gt;
-&lt;ar&gt;وَزْنَكَ، فَيَقُولُ: يَا رَبِّ مَا هَذِهِ الْبِطَاقَةُ مَعَ هَذِهِ السِّجِلَّاتِ؟ فَيَقُولُ: إِنَّكَ لَا تُظْلَمُ، قَالَ: فَتُوضَعُ السِّجِلَّاتُ فِي كِفَّةٍ، وَالْبِطَاقَةُ فِي كِفَّةٍ، فَطَاشَتِ السِّجِلَّاتُ وَثَقُلَتِ الْبِطَاقَةُ؛ فَلَا يَثْقُلُ مَعَ اسْمِ اللهِ شَيْءٌ .&lt;/ar&gt;
+&lt;ar&gt;عَنْ عَبْدِ اللَّهِ بْنِ عَمْرٍو قَالَ: قَالَ رَسُولُ اللهِ ﷺ : «إِنَّ اللَّهَ سَيُخَلَّصُ رَجُلًا مِنْ أُمَّتِي عَلَى رُءُوسِ الْخَلَائِقِ يَوْمَ الْقِيَامَةِ، فَيَنْشُرُ عَلَيْهِ تِسْعَةً وَتِسْعِينَ سِجِلًا، كُلُّ سِجِلٌ مِثْلَ مَدَّ الْبَصَرِ ، ثُمَّ يَقُولُ أَتُنْكِرُ مِنْ هَذَا شَيْئًا أَظْلَمَكَ كَتَبَتِي الْحَافِظُونَ؟ فَيَقُولُ: لَا يَا رَبِّ فَيَقُولُ: أَفَلَكَ عُذْرُ؟ قَالَ: لَا يَا رَبِّ فَيَقُولُ : بَلَى؛ إِنَّ لَكَ عِنْدَنَا حَسَنَةً، وَإِنَّهُ لَا ظُلْمَ عَلَيْكَ الْيَوْمَ، فَتُخْرَجُ بِطَاقَةٌ فِيهَا: أَشْهَدُ أَنْ لَا إِلَهَ إِلَّا اللهُ، وَأَنَّ مُحَمَّدًا عَبْدُهُ وَرَسُولُهُ، فَيَقُولُ: احْضُرْ وَزْنَكَ، فَيَقُولُ: يَا رَبِّ مَا هَذِهِ الْبِطَاقَةُ مَعَ هَذِهِ السِّجِلَّاتِ؟ فَيَقُولُ: إِنَّكَ لَا تُظْلَمُ، قَالَ: فَتُوضَعُ السِّجِلَّاتُ فِي كِفَّةٍ، وَالْبِطَاقَةُ فِي كِفَّةٍ، فَطَاشَتِ السِّجِلَّاتُ وَثَقُلَتِ الْبِطَاقَةُ؛ فَلَا يَثْقُلُ مَعَ اسْمِ اللهِ شَيْءٌ .&lt;/ar&gt;
 &lt;p&gt;আব্দুল্লাহ ইবনু আমর (রাঃ) বলেন, রাসূলুল্লাহ (ﷺ) বলেছেন, 'কিয়ামতের দিন এমন এক ব্যক্তিকে জনসম্মুখে উপস্থিত করা হবে, যার আমলনামা খোলা হবে নিরানব্বই ভলিয়মে এবং প্রতি ভলিয়ম বিস্তীর্ণ হবে দৃষ্টিসীমা পর্যন্ত। অতঃপর আল্লাহ তাআলা তাকে জিজ্ঞাসা করবেন, আচ্ছা বলো দেখি, তুমি এর কোনো একটিকে অস্বীকার করতে পারবে? অথবা আমার লিখক ফেরেশতাগণ কি তোমার প্রতি জুলুম করেছে? সে বলবে, না। হে আমার রব! আল্লাহ তাআলা জিজ্ঞাসা করবেন, তবে কি তোমার পক্ষ হতে কোনো ওযর পেশ করার আছে? সে বলবে, না; হে আমার রব! তখন আল্লাহ বলবেন, হ্যাঁ, তোমার একটি নেকী আমার নিকট রক্ষিত আছে। তুমি নিশ্চিত জেনে রাখ, আজ তোমার প্রতি কোনো জুলুম বা অবিচার করা হবে না। এরপর এক টুকরা কাগজ বের করা হবে, যাতে লিখা আছে, &lt;ar&gt;أَشْهَدُ أَنْ لَا إِلَهَ إِلَّا اللَّهُ وَأَنَّ مُحَمَّدًا رَّسُوْلُ اللَّهِ&lt;/ar&gt; [অর্থাৎ আমি সাক্ষ্য দিচ্ছি যে, আল্লাহ ছাড়া কোনো ইলাহ, (মা'বুদ) নেই এবং মুহাম্মাদ (ﷺ) তাঁর বান্দা ও রাসূল]। অতঃপর আল্লাহ তাকে বলবেন, তোমার আমলের ওজন দেখার জন্য উপস্থিত হও। তখন সে বলবে, হে আমার রব! ঐ সমস্ত বিরাট বিরাট দফতরের মুকাবিলায় এই এক টুকরা কাগজের মূল্যই বা কী আছে? তখন আল্লাহ বলবেন, তোমার উপর কোনো অবিচার করা হবে না। নবী করীম (ﷺ) বলেন, অতঃপর ঐ সমস্ত দফতরগুলো এক পাল্লায় এবং এই কাগজের টুকরাখানি আরেক পাল্লায় থাকবে। কাগজের টুকরা যে পাল্লায় থাকবে তা ভারী হয়ে নিচের দিকে ঝুঁকে থাকবে। মোটকথা, আল্লাহর নামের সাথে অন্য কোনো জিনিস ওজনই হতে পারবে না' (তিরমিযী, হা/২৬৩৯; ইবনু হিব্বান, হা/২২৫; মিশকাত, হা/৫৫৫৯)।&lt;/p&gt;
 &lt;ar&gt;عَنْ عَدِيِّ بْنِ حَاتِمٍ قَالَ : قَالَ رَسُولُ اللهِ ﷺ : «مَا مِنْكُمْ مِنْ أَحَدٍ إِلَّا سَيُكَلِّمُهُ رَبُّهُ، لَيْسَ بَيْنَهُ وَبَيْنَهُ تُرْجُمَانُ وَلَا حِجَابٌ يَحْجُبُهُ، فَيَنْظُرُ أَيْمَنَ مِنْهُ، فَلَا يَرَى إِلَّا مَا قَدَّمَ مِنْ عَمَلِهِ، وَيَنْظُرُ أَشْأَمَ مِنْهُ فَلَا يَرَى إِلَّا مَا قَدَّمَ، وَيَنْظُرُ بَيْنَ يَدَيْهِ فَلَا يَرَى إِلَّا النَّارَ تِلْقَاءَ وَجْهِهِ، فَاتَّقُوا النَّارَ وَلَوْ بِشِقِّ تَمْرَةٍ».&lt;/ar&gt;
-&lt;p&gt;আদী ইবনু হাতেম (রাঃ) হতে বর্ণিত, তিনি বলেন, রাসূলুল্লাহ (ﷺ) বলেছেন, তোমাদের মধ্যে এমন কেউ নেই, যার সাথে তার রব কথাবার্তা&lt;/p&gt;
-&lt;p&gt;বলবেন না। তার ও তার রবের মধ্যে কোনো দোভাষী এবং এমন কোনো পর্দা থাকবে না, যা তাকে আড়াল করে রাখবে। সে তার ডানে তাকাবে, তখনও পূর্বে প্রেরিত আমল ছাড়া আর কিছুই দেখতে পাবে না। আবার বামে তাকাবে, তখনও পূর্ব প্রেরিত আমল ছাড়া আর কিছুই দেখতে পাবে না। আর সম্মুখের দিকে তাকালে জাহান্নাম ছাড়া আর কিছুই দেখতে পাবে না। যা একেবারে চেহারার সম্মুখে অবস্থিত। সুতরাং খেজুর ছালের বিনিময়ে হলেও জাহান্নাম হতে বাঁচতে চেষ্টা করো' (ছহীহ বুখারী, হা/৭৫১২; মিশকাত, হা/৫৫৫০)।&lt;/p&gt;
+&lt;p&gt;আদী ইবনু হাতেম (রাঃ) হতে বর্ণিত, তিনি বলেন, রাসূলুল্লাহ (ﷺ) বলেছেন, তোমাদের মধ্যে এমন কেউ নেই, যার সাথে তার রব কথাবার্তা বলবেন না। তার ও তার রবের মধ্যে কোনো দোভাষী এবং এমন কোনো পর্দা থাকবে না, যা তাকে আড়াল করে রাখবে। সে তার ডানে তাকাবে, তখনও পূর্বে প্রেরিত আমল ছাড়া আর কিছুই দেখতে পাবে না। আবার বামে তাকাবে, তখনও পূর্ব প্রেরিত আমল ছাড়া আর কিছুই দেখতে পাবে না। আর সম্মুখের দিকে তাকালে জাহান্নাম ছাড়া আর কিছুই দেখতে পাবে না। যা একেবারে চেহারার সম্মুখে অবস্থিত। সুতরাং খেজুর ছালের বিনিময়ে হলেও জাহান্নাম হতে বাঁচতে চেষ্টা করো' (ছহীহ বুখারী, হা/৭৫১২; মিশকাত, হা/৫৫৫০)।&lt;/p&gt;
 &lt;ar&gt;عَنْ أَبِي سَعِيدٍ الْخُدْرِي  قَالَ قَالَ رَسُولُ اللهِ   ( وَالَّذِي نَفْسِي بِيَدِهِ لَا تَقُومُ السَّاعَةُ حَتَّى تُكَلِّمَ السَّاعَةُ حَتَّى تُكَلِّمَ السَّبَاعُ الإِنْسَ وَحَتَّى تُكَلِّمَ الرَّجُلَ عَذَبَةُ سَوْطِهِ وَشِرَاكُ نَعْلِهِ وَتُخْبِرَهُ فَخِذْهُ بِمَا أَحْدَثَ أَهْلُهُ مِنْ بَعْدِهِ ».&lt;/ar&gt;
 &lt;p&gt;আবু সাঈদ খুদরী (রাঃ) বলেন, রাসূলুল্লাহ (ﷺ) বলেছেন, 'সেই মহান সত্তার কসম, যার হাতে আমার প্রাণ! সেই সময় পর্যন্ত কিয়ামত কায়েম হবে না যে পর্যন্ত না হিংস্র পশু মানুষের সাথে কথা বলবে এবং যে পর্যন্ত না কারও চাবুক তার সাথে কথা বলবে, তার জুতার ফিতা তার সাথে কথা বলবে। আর তার উরু তাকে জানিয়ে দিবে যে, তার অনুপস্থিতিতে তার স্ত্রী কী করেছে' (তিরমিযী, হা/২১৮১; মিশকাত, হা/৫৪৫৯)।&lt;/p&gt;
 &lt;ar&gt;عَنْ بَهِزِ بْنِ حَكِيمٍ عَنْ أَبِيْهِ عَنْ جَدِّهِ عَنِ النَّبِيِّ ﷺ قَالَ: «إِنَّكُمْ تُدْعَوْنَ مُقَدَّمُ عَلَى أَفْوَاهِكُمْ بِالْقِدَامِ، فَأَوَّلُ مَا يُسْأَلُ عَنْ أَحَدِكُمْ فَخِدْهُ وَكَفُهُ».&lt;/ar&gt;
@@ -585,8 +582,7 @@
 &lt;ar&gt;عَنْ خَوْلَةَ بِنْتِ قَيْسٍ له قَالَتْ: سَمِعْتُ رَسُولَ اللهِ ﷺ يَقُولُ: «إِنَّ هَذِهِ الْمَالَ خَضِرَةٌ حُلْوَةٌ، فَمَنْ أَصَابَهُ بِحَقِّهِ بُورِكَ لَهُ فِيهِ، وَرُبَّ مُتَخَوِّضٍ فِيمَا شَاءَتْ بِهِ نَفْسُهُ مِنْ مَالِ اللَّهِ وَرَسُولِهِ لَيْسَ لَهُ يَوْمَ الْقِيَامَةِ إِلَّا النَّارُ».&lt;/ar&gt;
 &lt;p&gt;খাওলা বিনতে কায়স (রাঃ) হতে বর্ণিত, তিনি বলেন, আমি রাসূল (ﷺ)-কে বলতে শুনেছি, তিনি বলেন, 'নিশ্চয়ই এই পার্থিব সম্পদ শ্যামল ও সুমিষ্ট (অর্থাৎ আকর্ষণীয়) তবে যেই ব্যক্তি ন্যায়ভাবে প্রাপ্ত হয় তাতে তার বরকত হয়। আবার বহু লোক এমনও আছে, যে আল্লাহ ও তাঁর রাসূলের সম্পদে (অর্থাৎ গনীমতের মালে) যথেচ্ছা তসরূপ করে, তার জন্য কিয়ামতের দিন জাহান্নামের আগুন ব্যতীত আর কিছুই না' (তিরমিযী, হা/২৩৭৭; মিশকাত, হা/৪০১৭)।&lt;/p&gt;
 &lt;ar&gt;عَنْ أَبِي هُرَيْرَةَ هُ قَالَ: قَامَ فِينَا رَسُولُ اللهِ ﷺ ذَاتَ يَوْمٍ، فَذَكَرَ الْغُلُولَ، فَعَظَّمَهُ وَعَظَّمَ أَمْرَهُ، ثُمَّ قَالَ: «لَا أُلْفِيَنَّ أَحَدَكُمْ يَجِيءُ يَوْمَ الْقِيَامَةِ عَلَى رَقَبَتِهِ بَعِيرٌ لَهُ رُغَاءُ يَقُولُ: يَا رَسُولَ اللَّهِ! أَغِثْنِي، فَأَقُولُ لَا أَمْلِكُ لَكَ شَيْئًا، قَدْ أَبْلَغْتُكَ. لَا أُلْفِيَنَّ أَحَدَكُمْ يَجِيءُ يَوْমَ الْقِيَامَةِ عَلَى رَقَبَتِهِ فُرْسُ لَهُ حَمْحَمَةٌ، فَيَقُولُ: يَا رَسُولَ اللهِ أَغِثْنِي، فَأَقُولُ: لَا أَمْلِكُ لَكَ شَيْئًا، قَدْ أَبْلَغْتُكَ، لَا أُلْفِيَنَّ أَحَدَكُمْ يَجِيءُ يَوْমَ الْقِيَامَةِ عَلَى رَقَبَتِهِ شَاةٌ لَهَا ثُغَاءُ يَقُولُ: يَا رَسُولَ اللَّهِ أَغِثْنِي، فَأَقُولُ: لَا أَمْلِكُ لَكَ شَيْئًا قَدْ أَبْلَগْتُكَ. لَا أُلْفِيَنَّ أَحَدَكُمْ يَجِيءُ الْقِيَامَةِ عَلَى رَقَبَتِهِ نَفْسٌ لَهَا صِيَاحٌ، فَيَقُولُ : يَا رَسُولَ اللهِ أَغِثْنِي، فَأَقُولُ: لَا أَمْلِكُ لَكَ شَيْئًا، قَدْ أَبْلَغْتُكَ. لَا أُلْفِيَنَّ أَحَدَكُمْ يَجِيءُ يَوْমَ الْقِيَامَةِ عَلَى رَقَبَتِهِ رِقَاعٌ تَخْفُقُ، فَيَقُولُ: يَا رَسُولَ اللَّهِ أَغِثْنِي، فَأَقُولُ : لَا أَمْلِكُ لَكَ شَيْئًا، قَدْ أَبْلَغْتُكَ. لَا أُلْفِيَنَّ أَحَدَكُمْ يَجِيءُ يَوْمَ الْقِيَامَةِ عَلَى رَقَبَتِهِ صَامِتُ، فَيَقُولُ: يَا رَسُولَ اللهِ أَغِثْنِي، فَأَقُولُ: لَا أَمْلِكُ لَكَ شَيْئًا، قَدْ أَبْلَغْتُكَ»&lt;/ar&gt;
-&lt;p&gt;আবূ হুরায়রা (রাঃ) হতে বর্ণিত, তিনি বলেন, একদা নবী (ﷺ) আমাদের মাঝে বক্তব্য দেওয়ার জন্য দাঁড়ালেন, তিনি খিয়ানত সম্পর্কে বক্তব্য দিলেন এবং খিয়ানতের বিষয়টি খুব বড় করে পেশ করলেন। তারপর তিনি বললেন, 'কিয়ামতের দিন তোমাদের কাউকে আমি এমন অবস্থায় পাব যে, তার কাঁধের উপর উট চিৎকার করতে থাকবে। সে বলবে, হে আল্লাহর রাসূল! আমাকে রক্ষা&lt;/p&gt;
-&lt;p&gt;করুন। আমি বলব, আজ আল্লাহর সামনে তোমার জন্য সামান্য কিছু করার ক্ষমতা আমি রাখি না, যা পূর্বেই বলেছি। কিয়ামতের দিন আমি তোমাদের কাউকে এমন অবস্থায় পাব যে, তার কাঁধের উপর ঘোড়া চিৎকার করতে থাকবে। সে বলবে, হে আল্লাহর রাসূল! আমাকে রক্ষা করুন, আমি বলব, আজ আল্লাহর সামনে তোমার জন্য সামান্য কিছু করার ক্ষমতা আমার নেই, যা আমি পূর্বেই বলেছি। কিয়ামতের দিন আমি যেন তোমাদের কাউকে এই অবস্থায় দেখতে না পাই যে, সে কাঁধের উপর একটি ছাগল বহন করছে এবং আমাকে বলবে, আল্লাহর রাসূল আমাকে সাহায্য করুন। আর আমি বলব, আমি কিছুই করতে পারব না। আমি তো তোমাকে আল্লাহর বিধান পূর্বেই জানিয়ে দিয়েছি। কিয়ামতের দিন আমি যেন তোমাদের কাউকে এমন অবস্থায় দেখতে না পাই যে, সে নিজের কাঁধের উপর চিৎকাররত একটি মানুষ বহন করে নিয়ে আসবে আর আমাকে বলবে, হে আল্লাহর রাসূল! আমাকে সাহায্য করুন। আর আমি বলব, আজ আমি তোমার জন্য কিছুই করতে পারব না। আমি আল্লাহর বিধান তোমাকে পূর্বেই জানিয়ে দিয়েছি। কিয়ামতের দিন আমি যেন তোমাদের কাউকে এ অবস্থায় দেখতে না পাই যে, সে নিজের কাঁধের উপর কাপড় ইত্যাদির এক খণ্ড বহন করে নিয়ে আসছে। আর তা ভীষণভাবে তার কাঁধের উপর দুলছে, তখন সে আমাকে বলবে, হে আল্লাহর রাসূল! আমাকে সাহায্য করুন, আর আমি বলব, আমি তোমার জন্য কিছুই করতে পারব না। কিয়ামতে আমি যেন তোমাদের কাউকে এমন অবস্থায় না দেখতে পাই যে, সে নিজের কাঁধের উপর অচেতন সম্পদ (সোনা-চাঁদি) বহন করে নিয়ে আসছে। আর আমাকে বলবে, হে আল্লাহর রাসূল! আমাকে সাহায্য করুন। আর আমি বলব, আজ আমি তোমাকে কোনো সাহায্য করতে পারব না। আমি তো তোমাকে আল্লাহর বিধান পূর্বেই জানিয়ে দিয়েছি' (ছহীহ মুসলিম, হা/১৮৩১; মিশকাত, হা/৩৯৯৬)।&lt;/p&gt;
+&lt;p&gt;আবূ হুরায়রা (রাঃ) হতে বর্ণিত, তিনি বলেন, একদা নবী (ﷺ) আমাদের মাঝে বক্তব্য দেওয়ার জন্য দাঁড়ালেন, তিনি খিয়ানত সম্পর্কে বক্তব্য দিলেন এবং খিয়ানতের বিষয়টি খুব বড় করে পেশ করলেন। তারপর তিনি বললেন, 'কিয়ামতের দিন তোমাদের কাউকে আমি এমন অবস্থায় পাব যে, তার কাঁধের উপর উট চিৎকার করতে থাকবে। সে বলবে, হে আল্লাহর রাসূল! আমাকে রক্ষা করুন। আমি বলব, আজ আল্লাহর সামনে তোমার জন্য সামান্য কিছু করার ক্ষমতা আমি রাখি না, যা পূর্বেই বলেছি। কিয়ামতের দিন আমি তোমাদের কাউকে এমন অবস্থায় পাব যে, তার কাঁধের উপর ঘোড়া চিৎকার করতে থাকবে। সে বলবে, হে আল্লাহর রাসূল! আমাকে রক্ষা করুন, আমি বলব, আজ আল্লাহর সামনে তোমার জন্য সামান্য কিছু করার ক্ষমতা আমার নেই, যা আমি পূর্বেই বলেছি। কিয়ামতের দিন আমি যেন তোমাদের কাউকে এই অবস্থায় দেখতে না পাই যে, সে কাঁধের উপর একটি ছাগল বহন করছে এবং আমাকে বলবে, আল্লাহর রাসূল আমাকে সাহায্য করুন। আর আমি বলব, আমি কিছুই করতে পারব না। আমি তো তোমাকে আল্লাহর বিধান পূর্বেই জানিয়ে দিয়েছি। কিয়ামতের দিন আমি যেন তোমাদের কাউকে এমন অবস্থায় দেখতে না পাই যে, সে নিজের কাঁধের উপর চিৎকাররত একটি মানুষ বহন করে নিয়ে আসবে আর আমাকে বলবে, হে আল্লাহর রাসূল! আমাকে সাহায্য করুন। আর আমি বলব, আজ আমি তোমার জন্য কিছুই করতে পারব না। আমি আল্লাহর বিধান তোমাকে পূর্বেই জানিয়ে দিয়েছি। কিয়ামতের দিন আমি যেন তোমাদের কাউকে এ অবস্থায় দেখতে না পাই যে, সে নিজের কাঁধের উপর কাপড় ইত্যাদির এক খণ্ড বহন করে নিয়ে আসছে। আর তা ভীষণভাবে তার কাঁধের উপর দুলছে, তখন সে আমাকে বলবে, হে আল্লাহর রাসূল! আমাকে সাহায্য করুন, আর আমি বলব, আমি তোমার জন্য কিছুই করতে পারব না। কিয়ামতে আমি যেন তোমাদের কাউকে এমন অবস্থায় না দেখতে পাই যে, সে নিজের কাঁধের উপর অচেতন সম্পদ (সোনা-চাঁদি) বহন করে নিয়ে আসছে। আর আমাকে বলবে, হে আল্লাহর রাসূল! আমাকে সাহায্য করুন। আর আমি বলব, আজ আমি তোমাকে কোনো সাহায্য করতে পারব না। আমি তো তোমাকে আল্লাহর বিধান পূর্বেই জানিয়ে দিয়েছি' (ছহীহ মুসলিম, হা/১৮৩১; মিশকাত, হা/৩৯৯৬)।&lt;/p&gt;
 &lt;ar&gt;عَنْ أَبِي هُرَيْرَةَ قَالَ: «أَهْدَى رَجُلٌ لِرَسُولِ اللهِ ﷺ غُلَامًا يُقَالُ لَهُ: مِدْعَمُ فَبَيْنَمَا مِدْعَمُ يَحُطُّ رَحْلًا لِرَسُولِ اللهِ ﷺ إِذْ أَصَابَهُ سَهْمُ عَائِرٌ فَقَتَلَهُ، فَقَالَ النَّاسُ: هَنِيئًا لَهُ الْجَنَّةُ، فَقَالَ رَسُولُ اللهِ ﷺ : كَلَّا ، وَالَّذِي نَفْسِي بِيَدِهِ إِنَّ الشَّمْلَةَ الَّتِي أَخَذَهَا يَوْمَ خَيْبَرَ مِنَ الْمَغَانِمِ لَمْ تُصِبْهَا الْمَقَاسِمُ، لَتَشْتَعِلُ عَلَيْهِ نَارًا فَلَمَّا سَمِعَ ذَلِكَ النَّاسُ جَاءَ رَجُلٌ بِشِرَاكٍ، أَوْ شِرَاكَيْنِ إِلَى النَّبِيِّ ﷺ فَقَالَ: شِرَاكَ مِنْ نَارٍ، أَوْ شِرَاكَانِ مِنْ نَارٍ» .&lt;/ar&gt;
 &lt;p&gt;আবূ হুরায়রা (রাঃ) বলেন, মিদআম নামে একটি গোলাম রাসূল (ﷺ)-কে হাদিয়া দিয়েছিল। মিদআম এক সময় রাসূল (ﷺ)-এর উটের পিঠের হাওদা নামাচ্ছিল এমতাবস্থায় একটি তীর এসে তাকে লাগে এবং সে মারা যায়। ছাহাবীগণ বলেন, তার জন্য জান্নাত। রাসূল (ﷺ) বললেন, কখনই নয়।&lt;/p&gt;
 &lt;p&gt;আল্লাহর কসম, নিশ্চয়ই ঐ চাদরটি যেটি সে 'খায়বার'-এর গনীমত বণ্টন করার পূর্বে আত্মসাৎ করেছিল সে চাদরটি জাহান্নামের আগুন তার উপর উত্তেজিত করছে। এ কথা শুনে একজন লোক একটি জুতার ফিতা বা দুটি জুতার ফিতা রাসূল (ﷺ)-এর নিকট নিয়ে আসল। রাসূল (ﷺ) বললেন, একটি বা দুটি জুতার ফিতা আত্মসাৎ করলেও জাহান্নামে যাবে (ছহীহ বুখারী, হা/৬৭০৭; ছহীহ মুসলিম, হা/১১৫; মিশকাত, হা/৩৯৯৭)।&lt;br&gt;&lt;br&gt;এই হাদীছসমূহ দ্বারা প্রমাণিত হয় যে, আত্মসাৎকৃত বস্তু ক্ষুদ্র হলেও তার পরিণাম জাহান্নাম।&lt;/p&gt;
@@ -626,8 +622,7 @@
 &lt;ar&gt;يَا أَيُّهَا الرُّسُلُ كُلُوا مِنَ الطَّيِّبَاتِ وَاعْمَلُوا صَالِحًا إِنِّي بِمَا تَعْمَلُوْنَ عَلِيمٌ)&lt;/ar&gt;
 &lt;p&gt;'হে রাসূলগণ! তোমরা পবিত্র বস্তু হতে আহার করো ও সৎকর্ম করো; তোমরা যা কর সে সম্বন্ধে আমি অবগত' (আল-মুমিনূন, ২৩/৫১)।&lt;/p&gt;
 &lt;ar&gt;عَنْ أَبِي هُرَيْرَةَ هُ قَالَ: «قَالَ رَسُولُ اللهِ اللهِ : إِنَّ اللهَ طَيِّبُ لَا يَقْبَلُ إِلَّا طَيِّبًا، وَأَنَّ اللَّهَ أَمَرَ الْمُؤْمِنِينَ بِمَا أَمَرَ بِهِ الْمُرْسَلِينَ ثُمَّ ذَكَرَ الرَّجُلَ يُطِيلُ السَّفَرَ، أَشْعَثَ، أَغْبَرَ، يَمُدُّ يَدَيْهِ إِلَى السَّمَاءِ: يَا رَبِّ يَا رَبِّ وَمَطْعَمُهُ حَرَامٌ ، وَمَشْرَبُهُ حَرَامٌ ، وَمَلْبَسُهُ حَرَামٌ، وَغُذَّيَ بِالْحَرَامِ، فَأَنَّى يُسْتَجَابُ لِذَلِكَ؟».&lt;/ar&gt;
-&lt;p&gt;আবু হুরায়রা (রাঃ) বলেন, রাসূল (ﷺ) বলেছেন, 'নিশ্চয়ই আল্লাহ পবিত্র, তিনি পবিত্র ছাড়া গ্রহণ করেন না। (এবং সর্বক্ষেত্রে পাক-পবিত্রতার আদেশই তিনি করেছেন। সেই সম্পর্কে) আল্লাহ রাসূলগণকে যে আদেশ করেছেন, মুমিনগণকেও সেই আদেশই করেছেন। অতঃপর রাসূল (ﷺ) উল্লেখ করলেন, এক ব্যক্তি দূর-দূরান্তের সফর করছে। তার মাথার চুল এলোমেলো, শরীরে ধূলা-বালি। এমতাবস্থায় ঐ ব্যক্তি উভয় হস্ত আসমানের দিকে উঠিয়ে কাতর&lt;/p&gt;
-&lt;p&gt;স্বরে হে প্রভু! হে প্রভু! বলে ডাকছে। কিন্তু তার খাদ্য হারাম, তার পানীয় হারাম, তার পোশাক হারাম, তার জীবিকা নির্বাহ হারাম, কীভাবে তার দু'আ কবুল হবে' (ছহীহ মুসলিম, হা/১০১৫; তিরমিযী, হা/২৯৮৯; মিশকাত হা/২৭৬০)।&lt;/p&gt;
+&lt;p&gt;আবু হুরায়রা (রাঃ) বলেন, রাসূল (ﷺ) বলেছেন, 'নিশ্চয়ই আল্লাহ পবিত্র, তিনি পবিত্র ছাড়া গ্রহণ করেন না। (এবং সর্বক্ষেত্রে পাক-পবিত্রতার আদেশই তিনি করেছেন। সেই সম্পর্কে) আল্লাহ রাসূলগণকে যে আদেশ করেছেন, মুমিনগণকেও সেই আদেশই করেছেন। অতঃপর রাসূল (ﷺ) উল্লেখ করলেন, এক ব্যক্তি দূর-দূরান্তের সফর করছে। তার মাথার চুল এলোমেলো, শরীরে ধূলা-বালি। এমতাবস্থায় ঐ ব্যক্তি উভয় হস্ত আসমানের দিকে উঠিয়ে কাতর স্বরে হে প্রভু! হে প্রভু! বলে ডাকছে। কিন্তু তার খাদ্য হারাম, তার পানীয় হারাম, তার পোশাক হারাম, তার জীবিকা নির্বাহ হারাম, কীভাবে তার দু'আ কবুল হবে' (ছহীহ মুসলিম, হা/১০১৫; তিরমিযী, হা/২৯৮৯; মিশকাত হা/২৭৬০)।&lt;/p&gt;
 &lt;ar&gt;عَنْ أَبِي هُرَيْرَةَ الله قَالَ: قَالَ رَسُولُ اللهِ ﷺ : يَأْتِي عَلَى الْمَرْءِ زَمَانٌ لَا يُبَالِي الْمَرْءُ مَا أَخَذَ مِنْهُ، أَمِنَ الْحَلَالِ أَمْ مِنَ الْحَرَامِ».&lt;/ar&gt;
 &lt;p&gt;আবু হুরায়রা (রাঃ) বলেন, রাসূল (ﷺ) বলেছেন, 'মানুষের সম্মুখে এমন এক যুগ আসবে যে, কেউ পরওয়া করবে না কী উপায়ে মাল অর্জন করল; হারাম না হালাল উপায়ে' (ছহীহ বুখারী, হা/২০৫৯; মিশকাত, হা/২৭৬১)।&lt;/p&gt;
 &lt;ar&gt;وَعَنِ النُّعْمَانِ بْنِ بَشِيرٍ قَالَ: قَالَ رَسُولُ اللهِ ﷺ : الْحَلَالُ بَيِّنُ وَالْحَرَامُ بَيِّنٌ، وَبَيْنَهُمَا مُشْتَبِهَاتٌ لَا يَعْلَمُهُنَّ كَثِيرٌ مِنَ النَّاسِ، فَمَنِ اتَّقَى الشُّبَهَاتِ اسْتَبْرَأَ لِدِينِهِ وَعِرْضِهِ، وَمَنْ وَقَعَ فِي الْحَرَامِ كَالرَّاعِي يَرْعَى حَوْلَ الْحِمَى يُوشِكُ أَنْ يَرْتَعَ فِيهِ، أَلَا وَإِنَّ لِكُلِّ مَلِكٍ حِمّى أَلَا وَإِنَّ حِمَى اللَّهِ مَحَارِمُهُ، أَلَا وَإِنَّ فِي الْجَسَدِ مُضْغَةً إِذَا صَلُحَتْ صَلَحَ الْجُسَدُ كُلُّهُ، وَإِذَا فَسَدَتْ فَسَدَ الْجَسَدُ كُلُّهُ، أَلَا وَهِيَ الْقَلْبُ».&lt;/ar&gt;
@@ -663,8 +658,7 @@
 &lt;p&gt;আব্দুল্লাহ ইবনু আমর (রাঃ) হতে বর্ণিত, তিনি বলেন, রাসূলুল্লাহ (ﷺ) বলেছেন, 'যাকাতের মাল ধনীদের জন্য হালাল নয়, সুস্থ সবলদের (খেটে খেতে সক্ষম) জন্যও নয়' (আবূ দাউদ, হা/১৬৩৪; তিরমিযী, হা/৬৫২; মিশকাত, হা/১৮৩০)।&lt;br&gt;&lt;br&gt;এই হাদীছ প্রমাণ করে, যাদের কাজ করে খাওয়ার সামর্থ্য আছে তাদের জন্য ছাদাকা খাওয়া জায়েয নয়।&lt;/p&gt;
 &lt;ar&gt;عَنْ عُبَيْدِ اللَّهِ بْنِ عَدِيِّ بْنِ الْخِيَارِ قَالَ: «أَخْبَرَنِي رَجُلَانِ أَنَّهُمَا أَتَيَا النَّبِيَّ ﷺ وَهُوَ فِي حَجَّةِ الْوَدَاعِ، وَهُوَ يُقَسِّمُ الصَّدَقَةَ فَسَأَلَاهُ مِنْهَا، فَرَفَعَ فِينَا النَّظَرَ، وَخَفَضَهُ فَرَآنَا جَلْدَيْنِ، فَقَالَ: " إِنْ شِئْتُمَا أَعْطَيْتُكুমَا وَلَا حَظٍّ فِيهَا لِغَنِيٌّ وَلَا لِقَوِيٌّ مُكْتَسِبٍ» ".&lt;/ar&gt;
 &lt;p&gt;উবায়দুল্লাহ ইবনু আদী ইবনু খিয়ার (রাঃ) হতে বর্ণিত, তিনি বলেন, আমাকে দু'ব্যক্তি জানিয়েছেন যে, বিদায় হজ্জে মানুষের মধ্যে যাকাতের মাল বণ্টন করার সময় তারা উভয়ে নবী (ﷺ)-এর কাছে উপস্থিত ছিলেন। তারা এ মালের কিছু অংশ নেবার জন্য আগ্রহ দেখান। দুজন বলেন, রাসূলুল্লাহ (ﷺ) (যাকাত নেবার আগ্রহ দেখে) আমাদের মাথা থেকে পা পর্যন্ত চোখ বুলালেন। আমাদের সুস্থ সবল দেখে বললেন, তোমরা যাকাত নিতে চাইলে আমি দিতে পারি। (কিন্তু মনে রাখবে,) ছাদাকা ও যাকাতের সম্পদে ধনীদের কোনো অংশ নেই। আর সুস্থ সবল এবং পরিশ্রম করতে সক্ষম লোকদের জন্য ছাদাকা ও যাকাত নয়' (আবু দাউদ, হা/১৬৩৩; নাসাঈ, হা/২৫৯৮; মিশকাত, হা/১৮৩২)।&lt;/p&gt;
-&lt;ar&gt;عَنْ قَبِيصَةَ بْنِ مُخَارِقٍ قَالَ: تَحَمَّلْتُ حَمَالَةً، فَأَتَيْتُ رَسُولَ اللَّهِ ﷺ أَسْأَلُهُ فِيهَا، فَقَالَ: " أَقِمْ حَتَّى تَأْتِيَنَا الصَّدَقَةُ، فَنَأْمُرَ لَكَ بِهَا " ، ثُمَّ قَالَ: " يَا قَبِيصَةُ إِنَّ الْمَسْأَلَةَ لَا تَحِلُّ إِلَّا لِأَحَدِ ثَلَاثَةٍ : رَجُلٍ تَحَمَّلَ حَمَالَةٌ فَحَلَّتْ لَهُ الْمَسْأَلَةُ حَتَّى يُصِيبَهَا ثُمَّ يُمْسِكُ، وَرَجُلٍ أَصَابَتْهُ جَائِحَةُ اجْتَاحَتْ مَالَهُ، فَحَلَّتْ لَهُ الْمَسْأَلَةُ حَتَّى يُصِيبَ قِوَامًا مِنْ عَيْشٍ، أَوْ قَالَ سِدَادًا مِنْ عَيْشٍ، وَرَجُلٍ أَصَابَتْهُ فَاقَةٌ حَتَّى يَقُولَ ثَلَاثَةٌ مِنْ ذَوِي الْخِجَا مِنْ قَوْمِهِ: لَقَدْ أَصَابَتْ فُلَانًا فَاقَةٌ&lt;/ar&gt;
-&lt;ar&gt;فَحَلَّتْ لَهُ الْمَسْأَلَةُ حَتَّى يُصِيبَ قِوَامًا مِنْ عَيْشٍ ، أَوْ قَالَ سِدَادًا مِنْ عَيْشٍ، فَمَا سِوَاهُنَّ مِنَ الْمَسْأَلَةِ يَا قَبِيصَةُ سُحْتُ، يَأْكُلُهَا صَاحِبُهَا سُحْتًا».&lt;/ar&gt;
+&lt;ar&gt;عَنْ قَبِيصَةَ بْنِ مُخَارِقٍ قَالَ: تَحَمَّلْتُ حَمَالَةً، فَأَتَيْتُ رَسُولَ اللَّهِ ﷺ أَسْأَلُهُ فِيهَا، فَقَالَ: " أَقِمْ حَتَّى تَأْتِيَنَا الصَّدَقَةُ، فَنَأْمُرَ لَكَ بِهَا " ، ثُمَّ قَالَ: " يَا قَبِيصَةُ إِنَّ الْمَسْأَلَةَ لَا تَحِلُّ إِلَّا لِأَحَدِ ثَلَاثَةٍ : رَجُلٍ تَحَمَّلَ حَمَالَةٌ فَحَلَّتْ لَهُ الْمَسْأَلَةُ حَتَّى يُصِيبَهَا ثُمَّ يُمْسِكُ، وَرَجُلٍ أَصَابَتْهُ جَائِحَةُ اجْتَاحَتْ مَالَهُ، فَحَلَّتْ لَهُ الْمَسْأَلَةُ حَتَّى يُصِيبَ قِوَامًا مِنْ عَيْشٍ، أَوْ قَالَ سِدَادًا مِنْ عَيْشٍ، وَرَجُلٍ أَصَابَتْهُ فَاقَةٌ حَتَّى يَقُولَ ثَلَاثَةٌ مِنْ ذَوِي الْخِجَا مِنْ قَوْمِهِ: لَقَدْ أَصَابَتْ فُلَانًا فَاقَةٌ فَحَلَّتْ لَهُ الْمَسْأَلَةُ حَتَّى يُصِيبَ قِوَامًا مِنْ عَيْشٍ ، أَوْ قَالَ سِدَادًا مِنْ عَيْشٍ، فَمَا سِوَاهُنَّ مِنَ الْمَسْأَلَةِ يَا قَبِيصَةُ سُحْتُ، يَأْكُلُهَا صَاحِبُهَا سُحْتًا».&lt;/ar&gt;
 &lt;p&gt;কবীসা ইবনু মুখারিক্ক (রাঃ) হতে বর্ণিত, তিনি বলেন, আমি ঋণগ্রস্ত হয়ে রাসূলুল্লাহ (ﷺ)-এর কাছে এলাম। তার কাছে ঋণ আদায়ের জন্য কিছু চাইলাম। তিনি বললেন, অপেক্ষা করো। আমার কাছে যাকাতের মাল আসা পর্যন্ত আসলে তোমাকে কিছু দেবার জন্য বলে দেব। তারপর তিনি বললেন, কবীসা! শুধু তিন ধরনের ব্যক্তির জন্য কিছু চাওয়া জায়েয। প্রথমত, যে ব্যক্তি অপরের ঋণের জামিনদার। তবে বেশি চাইতে পারবে না। বরং যতটুকু ঋণ শোধের জন্য প্রয়োজন শুধু ততটুকু চাইবে। এরপর আর চাইবে না। দ্বিতীয়ত, ওই ব্যক্তি যে বিপদগ্রস্ত হয়ে পড়েছে (দুর্ভিক্ষ, প্লাবন ইত্যাদিতে)। তার সব ধন-সম্পদ ধ্বংস হয়েছে। তারও (শুধু খাবার ও পোশাকের জন্য) ততটুকু যাতে প্রয়োজন মিটে যায়। তার জীবনের জন্য অবলম্বন হয়ে যায়। তৃতীয়ত, ওই ব্যক্তি (যে ধনী, কিন্তু তার এমন কোনো কঠিন প্রয়োজন হয়ে পড়েছে যা মহল্লাবাসী জানে। যেমন ঘরের সব মালপত্র চুরি হয়ে গেছে অথবা অন্য কোনো দুর্ঘটনার কারণে মুখাপেক্ষী হয়ে পড়েছে)। (মহল্লার) তিনজন বুদ্ধিমান সচেতন লোক এ ব্যাপারে সাক্ষ্য দিবে যে, সত্যিই এ ব্যক্তি মুখাপেক্ষী। তার জন্যও সেই পরিমাণ (সাহায্য) চাওয়া জায়েয, যাতে তার প্রয়োজন মিটে। অথবা তিনি বলেছেন এর দ্বারা তার মুখাপেক্ষিতা ও অভাব দূর হয়, তার জীবনে একটি অবলম্বন আসে। হে ক্ববীসা! এ তিন প্রকারের 'চাওয়া' ছাড়া হালাল নয়। আর হারাম পন্থায় প্রাপ্ত মাল খাওয়া তার জন্য হারাম (ছহীহ মুসলিম, হা/১০৪৪; মিশকাত, হা/১৮৩৭)।&lt;/p&gt;&lt;/div&gt;</t>
         </is>
       </c>

</xml_diff>